<commit_message>
feat: add Boshlanish and Tugash times to Excel template
</commit_message>
<xml_diff>
--- a/admin/public/Darslar_Shabloni.xlsx
+++ b/admin/public/Darslar_Shabloni.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
   <si>
     <t>Guruh</t>
   </si>
@@ -22,6 +22,12 @@
     <t>Sana</t>
   </si>
   <si>
+    <t>Boshlanish</t>
+  </si>
+  <si>
+    <t>Tugash</t>
+  </si>
+  <si>
     <t>Mavzu</t>
   </si>
   <si>
@@ -44,6 +50,24 @@
   </si>
   <si>
     <t>YYYY-MM-DD formatida</t>
+  </si>
+  <si>
+    <t>09:00</t>
+  </si>
+  <si>
+    <t>14:00</t>
+  </si>
+  <si>
+    <t>Dars boshlanish vaqti</t>
+  </si>
+  <si>
+    <t>15:00</t>
+  </si>
+  <si>
+    <t>20:00</t>
+  </si>
+  <si>
+    <t>Dars tugash vaqti</t>
   </si>
   <si>
     <t>Rangtasvir asoslari</t>
@@ -425,16 +449,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" customWidth="1"/>
-    <col min="3" max="3" width="35.7109375" customWidth="1"/>
-    <col min="4" max="4" width="25.7109375" customWidth="1"/>
+    <col min="2" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="35.7109375" customWidth="1"/>
+    <col min="6" max="6" width="25.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -447,47 +471,71 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="C3" t="s">
         <v>13</v>
       </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
+      <c r="C4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>